<commit_message>
bayesian score script + xscan script + other
</commit_message>
<xml_diff>
--- a/02_Data_Analysis/data/Bayesian/MAGEA3_summary.xlsx
+++ b/02_Data_Analysis/data/Bayesian/MAGEA3_summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">confidence_level</t>
   </si>
@@ -36,6 +36,12 @@
   </si>
   <si>
     <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
   </si>
   <si>
     <t xml:space="preserve">Very Low</t>
@@ -395,19 +401,19 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>261</v>
+        <v>159</v>
       </c>
       <c r="C2" t="n">
-        <v>99.5</v>
+        <v>99.7</v>
       </c>
       <c r="D2" t="n">
-        <v>99.9</v>
+        <v>99.7</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="F2" t="n">
-        <v>90.9</v>
+        <v>98.8</v>
       </c>
       <c r="G2" t="n">
         <v>100</v>
@@ -418,22 +424,66 @@
         <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>1195</v>
+        <v>99</v>
       </c>
       <c r="C3" t="n">
-        <v>16.7</v>
+        <v>64.3</v>
       </c>
       <c r="D3" t="n">
-        <v>16.7</v>
+        <v>64.3</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>16.7</v>
+        <v>64.3</v>
       </c>
       <c r="G3" t="n">
-        <v>16.7</v>
+        <v>64.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E4"/>
+      <c r="F4" t="n">
+        <v>31</v>
+      </c>
+      <c r="G4" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1195</v>
+      </c>
+      <c r="C5" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>23.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>